<commit_message>
M5 step 3: corrected scores so they match the data in the project (UC2 human review, UC4/UC7 data readiness, UC8 effort)
</commit_message>
<xml_diff>
--- a/excel/AI_Use_Case_Prioritization.xlsx
+++ b/excel/AI_Use_Case_Prioritization.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/mac1/Desktop/app_projects/supplier-data-health-check/excel/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{63B5538F-E1B7-9742-950A-AF58CEFCBD4B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2DB7B6C1-D7CB-9B45-9F57-E598A5A875CA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="16260" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -811,7 +811,7 @@
         <v>1</v>
       </c>
       <c r="L3" s="2" t="s">
-        <v>52</v>
+        <v>87</v>
       </c>
     </row>
     <row r="4" spans="1:12" ht="32" x14ac:dyDescent="0.2">
@@ -878,7 +878,7 @@
         <v>5</v>
       </c>
       <c r="I5" s="2">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="J5" s="2">
         <v>1</v>
@@ -992,7 +992,7 @@
         <v>5</v>
       </c>
       <c r="I8" s="2">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="J8" s="2">
         <v>3</v>
@@ -1033,7 +1033,7 @@
         <v>2</v>
       </c>
       <c r="J9" s="2">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="K9" s="2">
         <v>5</v>

</xml_diff>

<commit_message>
M5 step 4: weighted score column (value 40%, data readiness 20%, inverted effort 20%, inverted risk 20%)
</commit_message>
<xml_diff>
--- a/excel/AI_Use_Case_Prioritization.xlsx
+++ b/excel/AI_Use_Case_Prioritization.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/mac1/Desktop/app_projects/supplier-data-health-check/excel/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2DB7B6C1-D7CB-9B45-9F57-E598A5A875CA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C4D541F6-A211-8E4A-A20A-5DBD74405714}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="16260" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="105" uniqueCount="88">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="106" uniqueCount="89">
   <si>
     <t>ID</t>
   </si>
@@ -298,6 +298,9 @@
   </si>
   <si>
     <t>Yes</t>
+  </si>
+  <si>
+    <t>Weighted score</t>
   </si>
 </sst>
 </file>
@@ -367,7 +370,11 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
+  <dxfs count="1">
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
@@ -381,9 +388,9 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="tblUseCases" displayName="tblUseCases" ref="A1:L9">
-  <autoFilter ref="A1:L9" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
-  <tableColumns count="12">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="tblUseCases" displayName="tblUseCases" ref="A1:M9">
+  <autoFilter ref="A1:M9" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
+  <tableColumns count="13">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="ID"/>
     <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="Use case"/>
     <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="Problem it solves"/>
@@ -396,6 +403,9 @@
     <tableColumn id="10" xr3:uid="{00000000-0010-0000-0000-00000A000000}" name="Effort (1-5)"/>
     <tableColumn id="11" xr3:uid="{00000000-0010-0000-0000-00000B000000}" name="Risk (1-5)"/>
     <tableColumn id="12" xr3:uid="{00000000-0010-0000-0000-00000C000000}" name="Human approval needed?"/>
+    <tableColumn id="13" xr3:uid="{5EA26752-C517-2B41-B7F3-9C6366B9BA98}" name="Weighted score" dataDxfId="0">
+      <calculatedColumnFormula>H2*40%+I2*20%+(6-J2)*20%+(6-K2)*20%</calculatedColumnFormula>
+    </tableColumn>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -686,7 +696,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:L9"/>
+  <dimension ref="A1:M9"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="6" customWidth="1"/>
@@ -700,7 +710,7 @@
     <col min="12" max="12" width="14" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" ht="48" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:13" ht="48" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -737,8 +747,11 @@
       <c r="L1" s="1" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="2" spans="1:12" ht="32" x14ac:dyDescent="0.2">
+      <c r="M1" s="1" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="2" spans="1:13" ht="32" x14ac:dyDescent="0.2">
       <c r="A2" s="2" t="s">
         <v>12</v>
       </c>
@@ -775,8 +788,12 @@
       <c r="L2" s="2" t="s">
         <v>87</v>
       </c>
-    </row>
-    <row r="3" spans="1:12" ht="32" x14ac:dyDescent="0.2">
+      <c r="M2">
+        <f t="shared" ref="M2:M9" si="0">H2*40%+I2*20%+(6-J2)*20%+(6-K2)*20%</f>
+        <v>3.4000000000000004</v>
+      </c>
+    </row>
+    <row r="3" spans="1:13" ht="32" x14ac:dyDescent="0.2">
       <c r="A3" s="2" t="s">
         <v>19</v>
       </c>
@@ -813,8 +830,12 @@
       <c r="L3" s="2" t="s">
         <v>87</v>
       </c>
-    </row>
-    <row r="4" spans="1:12" ht="32" x14ac:dyDescent="0.2">
+      <c r="M3">
+        <f t="shared" si="0"/>
+        <v>4.8</v>
+      </c>
+    </row>
+    <row r="4" spans="1:13" ht="32" x14ac:dyDescent="0.2">
       <c r="A4" s="2" t="s">
         <v>26</v>
       </c>
@@ -851,8 +872,12 @@
       <c r="L4" s="2" t="s">
         <v>87</v>
       </c>
-    </row>
-    <row r="5" spans="1:12" ht="32" x14ac:dyDescent="0.2">
+      <c r="M4">
+        <f t="shared" si="0"/>
+        <v>3.8</v>
+      </c>
+    </row>
+    <row r="5" spans="1:13" ht="32" x14ac:dyDescent="0.2">
       <c r="A5" s="2" t="s">
         <v>31</v>
       </c>
@@ -889,8 +914,12 @@
       <c r="L5" s="2" t="s">
         <v>52</v>
       </c>
-    </row>
-    <row r="6" spans="1:12" ht="32" x14ac:dyDescent="0.2">
+      <c r="M5">
+        <f t="shared" si="0"/>
+        <v>4.5999999999999996</v>
+      </c>
+    </row>
+    <row r="6" spans="1:13" ht="32" x14ac:dyDescent="0.2">
       <c r="A6" s="2" t="s">
         <v>36</v>
       </c>
@@ -927,8 +956,12 @@
       <c r="L6" s="2" t="s">
         <v>52</v>
       </c>
-    </row>
-    <row r="7" spans="1:12" ht="32" x14ac:dyDescent="0.2">
+      <c r="M6">
+        <f t="shared" si="0"/>
+        <v>4.2</v>
+      </c>
+    </row>
+    <row r="7" spans="1:13" ht="32" x14ac:dyDescent="0.2">
       <c r="A7" s="2" t="s">
         <v>42</v>
       </c>
@@ -965,8 +998,12 @@
       <c r="L7" s="2" t="s">
         <v>52</v>
       </c>
-    </row>
-    <row r="8" spans="1:12" ht="32" x14ac:dyDescent="0.2">
+      <c r="M7">
+        <f t="shared" si="0"/>
+        <v>5</v>
+      </c>
+    </row>
+    <row r="8" spans="1:13" ht="32" x14ac:dyDescent="0.2">
       <c r="A8" s="2" t="s">
         <v>47</v>
       </c>
@@ -1003,8 +1040,12 @@
       <c r="L8" s="2" t="s">
         <v>87</v>
       </c>
-    </row>
-    <row r="9" spans="1:12" ht="32" x14ac:dyDescent="0.2">
+      <c r="M8">
+        <f t="shared" si="0"/>
+        <v>3.0000000000000004</v>
+      </c>
+    </row>
+    <row r="9" spans="1:13" ht="32" x14ac:dyDescent="0.2">
       <c r="A9" s="2" t="s">
         <v>53</v>
       </c>
@@ -1040,6 +1081,10 @@
       </c>
       <c r="L9" s="2" t="s">
         <v>87</v>
+      </c>
+      <c r="M9">
+        <f t="shared" si="0"/>
+        <v>1.6</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
M5 step 5: raised UC6 risk to 3 (LLM summaries can invent numbers) and added RANK.EQ column
</commit_message>
<xml_diff>
--- a/excel/AI_Use_Case_Prioritization.xlsx
+++ b/excel/AI_Use_Case_Prioritization.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/mac1/Desktop/app_projects/supplier-data-health-check/excel/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C4D541F6-A211-8E4A-A20A-5DBD74405714}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3413DB38-0A67-D241-9B12-192F3C23F8BF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="16260" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="106" uniqueCount="89">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="107" uniqueCount="90">
   <si>
     <t>ID</t>
   </si>
@@ -301,6 +301,9 @@
   </si>
   <si>
     <t>Weighted score</t>
+  </si>
+  <si>
+    <t>Rank</t>
   </si>
 </sst>
 </file>
@@ -370,7 +373,10 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="1">
+  <dxfs count="2">
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
     <dxf>
       <numFmt numFmtId="0" formatCode="General"/>
     </dxf>
@@ -388,9 +394,9 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="tblUseCases" displayName="tblUseCases" ref="A1:M9">
-  <autoFilter ref="A1:M9" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
-  <tableColumns count="13">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="tblUseCases" displayName="tblUseCases" ref="A1:N9">
+  <autoFilter ref="A1:N9" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
+  <tableColumns count="14">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="ID"/>
     <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="Use case"/>
     <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="Problem it solves"/>
@@ -403,8 +409,11 @@
     <tableColumn id="10" xr3:uid="{00000000-0010-0000-0000-00000A000000}" name="Effort (1-5)"/>
     <tableColumn id="11" xr3:uid="{00000000-0010-0000-0000-00000B000000}" name="Risk (1-5)"/>
     <tableColumn id="12" xr3:uid="{00000000-0010-0000-0000-00000C000000}" name="Human approval needed?"/>
-    <tableColumn id="13" xr3:uid="{5EA26752-C517-2B41-B7F3-9C6366B9BA98}" name="Weighted score" dataDxfId="0">
+    <tableColumn id="13" xr3:uid="{5EA26752-C517-2B41-B7F3-9C6366B9BA98}" name="Weighted score" dataDxfId="1">
       <calculatedColumnFormula>H2*40%+I2*20%+(6-J2)*20%+(6-K2)*20%</calculatedColumnFormula>
+    </tableColumn>
+    <tableColumn id="14" xr3:uid="{F0605FC8-72E2-6648-91FF-7735AC24D597}" name="Rank" dataDxfId="0">
+      <calculatedColumnFormula>_xlfn.RANK.EQ(M2,$M$2:$M$9)</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
@@ -696,7 +705,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:M9"/>
+  <dimension ref="A1:N9"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="6" customWidth="1"/>
@@ -710,7 +719,7 @@
     <col min="12" max="12" width="14" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" ht="48" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:14" ht="48" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -750,8 +759,11 @@
       <c r="M1" s="1" t="s">
         <v>88</v>
       </c>
-    </row>
-    <row r="2" spans="1:13" ht="32" x14ac:dyDescent="0.2">
+      <c r="N1" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="2" spans="1:14" ht="32" x14ac:dyDescent="0.2">
       <c r="A2" s="2" t="s">
         <v>12</v>
       </c>
@@ -792,8 +804,12 @@
         <f t="shared" ref="M2:M9" si="0">H2*40%+I2*20%+(6-J2)*20%+(6-K2)*20%</f>
         <v>3.4000000000000004</v>
       </c>
-    </row>
-    <row r="3" spans="1:13" ht="32" x14ac:dyDescent="0.2">
+      <c r="N2">
+        <f t="shared" ref="N2:N9" si="1">_xlfn.RANK.EQ(M2,$M$2:$M$9)</f>
+        <v>6</v>
+      </c>
+    </row>
+    <row r="3" spans="1:14" ht="32" x14ac:dyDescent="0.2">
       <c r="A3" s="2" t="s">
         <v>19</v>
       </c>
@@ -834,8 +850,12 @@
         <f t="shared" si="0"/>
         <v>4.8</v>
       </c>
-    </row>
-    <row r="4" spans="1:13" ht="32" x14ac:dyDescent="0.2">
+      <c r="N3">
+        <f t="shared" si="1"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4" spans="1:14" ht="32" x14ac:dyDescent="0.2">
       <c r="A4" s="2" t="s">
         <v>26</v>
       </c>
@@ -876,8 +896,12 @@
         <f t="shared" si="0"/>
         <v>3.8</v>
       </c>
-    </row>
-    <row r="5" spans="1:13" ht="32" x14ac:dyDescent="0.2">
+      <c r="N4">
+        <f t="shared" si="1"/>
+        <v>5</v>
+      </c>
+    </row>
+    <row r="5" spans="1:14" ht="32" x14ac:dyDescent="0.2">
       <c r="A5" s="2" t="s">
         <v>31</v>
       </c>
@@ -918,8 +942,12 @@
         <f t="shared" si="0"/>
         <v>4.5999999999999996</v>
       </c>
-    </row>
-    <row r="6" spans="1:13" ht="32" x14ac:dyDescent="0.2">
+      <c r="N5">
+        <f t="shared" si="1"/>
+        <v>2</v>
+      </c>
+    </row>
+    <row r="6" spans="1:14" ht="32" x14ac:dyDescent="0.2">
       <c r="A6" s="2" t="s">
         <v>36</v>
       </c>
@@ -960,8 +988,12 @@
         <f t="shared" si="0"/>
         <v>4.2</v>
       </c>
-    </row>
-    <row r="7" spans="1:13" ht="32" x14ac:dyDescent="0.2">
+      <c r="N6">
+        <f t="shared" si="1"/>
+        <v>4</v>
+      </c>
+    </row>
+    <row r="7" spans="1:14" ht="32" x14ac:dyDescent="0.2">
       <c r="A7" s="2" t="s">
         <v>42</v>
       </c>
@@ -993,17 +1025,21 @@
         <v>1</v>
       </c>
       <c r="K7" s="2">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="L7" s="2" t="s">
-        <v>52</v>
+        <v>87</v>
       </c>
       <c r="M7">
         <f t="shared" si="0"/>
-        <v>5</v>
-      </c>
-    </row>
-    <row r="8" spans="1:13" ht="32" x14ac:dyDescent="0.2">
+        <v>4.5999999999999996</v>
+      </c>
+      <c r="N7">
+        <f t="shared" si="1"/>
+        <v>2</v>
+      </c>
+    </row>
+    <row r="8" spans="1:14" ht="32" x14ac:dyDescent="0.2">
       <c r="A8" s="2" t="s">
         <v>47</v>
       </c>
@@ -1044,8 +1080,12 @@
         <f t="shared" si="0"/>
         <v>3.0000000000000004</v>
       </c>
-    </row>
-    <row r="9" spans="1:13" ht="32" x14ac:dyDescent="0.2">
+      <c r="N8">
+        <f t="shared" si="1"/>
+        <v>7</v>
+      </c>
+    </row>
+    <row r="9" spans="1:14" ht="32" x14ac:dyDescent="0.2">
       <c r="A9" s="2" t="s">
         <v>53</v>
       </c>
@@ -1085,6 +1125,10 @@
       <c r="M9">
         <f t="shared" si="0"/>
         <v>1.6</v>
+      </c>
+      <c r="N9">
+        <f t="shared" si="1"/>
+        <v>8</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
M5 step 6: Matrix sheet (cross-sheet references) and value-vs-effort scatter chart with use-case labels
</commit_message>
<xml_diff>
--- a/excel/AI_Use_Case_Prioritization.xlsx
+++ b/excel/AI_Use_Case_Prioritization.xlsx
@@ -8,13 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/mac1/Desktop/app_projects/supplier-data-health-check/excel/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3413DB38-0A67-D241-9B12-192F3C23F8BF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D76D9421-045E-6444-8C06-913A80401EDB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="16260" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="16260" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Use Cases" sheetId="1" r:id="rId1"/>
-    <sheet name="Scoring Guide" sheetId="2" r:id="rId2"/>
+    <sheet name="Matrix" sheetId="3" r:id="rId2"/>
+    <sheet name="Scoring Guide" sheetId="2" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -34,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="107" uniqueCount="90">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="110" uniqueCount="91">
   <si>
     <t>ID</t>
   </si>
@@ -304,6 +305,9 @@
   </si>
   <si>
     <t>Rank</t>
+  </si>
+  <si>
+    <t>Business Value</t>
   </si>
 </sst>
 </file>
@@ -391,6 +395,1303 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
+  <c:lang val="en-US"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:chart>
+    <c:title>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="en-TR"/>
+        </a:p>
+      </c:txPr>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:plotArea>
+      <c:layout/>
+      <c:scatterChart>
+        <c:scatterStyle val="lineMarker"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>Matrix!$C$1</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Business Value</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="28575" cap="rnd">
+              <a:noFill/>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="circle"/>
+            <c:size val="5"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent1"/>
+              </a:solidFill>
+              <a:ln w="9525">
+                <a:solidFill>
+                  <a:schemeClr val="accent1"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:marker>
+          <c:dLbls>
+            <c:dLbl>
+              <c:idx val="0"/>
+              <c:tx>
+                <c:rich>
+                  <a:bodyPr/>
+                  <a:lstStyle/>
+                  <a:p>
+                    <a:fld id="{AE28D843-2E10-8D4B-B511-6E5BD9871D2E}" type="CELLRANGE">
+                      <a:rPr lang="en-US"/>
+                      <a:pPr/>
+                      <a:t>[CELLRANGE]</a:t>
+                    </a:fld>
+                    <a:endParaRPr lang="en-US"/>
+                  </a:p>
+                </c:rich>
+              </c:tx>
+              <c:showLegendKey val="0"/>
+              <c:showVal val="0"/>
+              <c:showCatName val="0"/>
+              <c:showSerName val="0"/>
+              <c:showPercent val="0"/>
+              <c:showBubbleSize val="0"/>
+              <c:extLst>
+                <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
+                  <c15:dlblFieldTable/>
+                  <c15:xForSave val="1"/>
+                  <c15:showDataLabelsRange val="1"/>
+                </c:ext>
+                <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                  <c16:uniqueId val="{00000001-89D1-E846-B27A-3DA1AEF5883E}"/>
+                </c:ext>
+              </c:extLst>
+            </c:dLbl>
+            <c:dLbl>
+              <c:idx val="1"/>
+              <c:tx>
+                <c:rich>
+                  <a:bodyPr/>
+                  <a:lstStyle/>
+                  <a:p>
+                    <a:fld id="{C5B6A356-D241-8F4B-896C-8B0132F7D7E1}" type="CELLRANGE">
+                      <a:rPr lang="en-US"/>
+                      <a:pPr/>
+                      <a:t>[CELLRANGE]</a:t>
+                    </a:fld>
+                    <a:endParaRPr lang="en-US"/>
+                  </a:p>
+                </c:rich>
+              </c:tx>
+              <c:showLegendKey val="0"/>
+              <c:showVal val="0"/>
+              <c:showCatName val="0"/>
+              <c:showSerName val="0"/>
+              <c:showPercent val="0"/>
+              <c:showBubbleSize val="0"/>
+              <c:extLst>
+                <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
+                  <c15:dlblFieldTable/>
+                  <c15:xForSave val="1"/>
+                  <c15:showDataLabelsRange val="1"/>
+                </c:ext>
+                <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                  <c16:uniqueId val="{00000002-89D1-E846-B27A-3DA1AEF5883E}"/>
+                </c:ext>
+              </c:extLst>
+            </c:dLbl>
+            <c:dLbl>
+              <c:idx val="2"/>
+              <c:tx>
+                <c:rich>
+                  <a:bodyPr/>
+                  <a:lstStyle/>
+                  <a:p>
+                    <a:fld id="{A192A440-33E3-4848-B253-46A9D2677265}" type="CELLRANGE">
+                      <a:rPr lang="en-US"/>
+                      <a:pPr/>
+                      <a:t>[CELLRANGE]</a:t>
+                    </a:fld>
+                    <a:endParaRPr lang="en-US"/>
+                  </a:p>
+                </c:rich>
+              </c:tx>
+              <c:showLegendKey val="0"/>
+              <c:showVal val="0"/>
+              <c:showCatName val="0"/>
+              <c:showSerName val="0"/>
+              <c:showPercent val="0"/>
+              <c:showBubbleSize val="0"/>
+              <c:extLst>
+                <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
+                  <c15:dlblFieldTable/>
+                  <c15:xForSave val="1"/>
+                  <c15:showDataLabelsRange val="1"/>
+                </c:ext>
+                <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                  <c16:uniqueId val="{00000003-89D1-E846-B27A-3DA1AEF5883E}"/>
+                </c:ext>
+              </c:extLst>
+            </c:dLbl>
+            <c:dLbl>
+              <c:idx val="3"/>
+              <c:tx>
+                <c:rich>
+                  <a:bodyPr/>
+                  <a:lstStyle/>
+                  <a:p>
+                    <a:fld id="{E2707DB1-2CC9-5046-B13E-9112D8CBEA8A}" type="CELLRANGE">
+                      <a:rPr lang="en-US"/>
+                      <a:pPr/>
+                      <a:t>[CELLRANGE]</a:t>
+                    </a:fld>
+                    <a:endParaRPr lang="en-US"/>
+                  </a:p>
+                </c:rich>
+              </c:tx>
+              <c:showLegendKey val="0"/>
+              <c:showVal val="0"/>
+              <c:showCatName val="0"/>
+              <c:showSerName val="0"/>
+              <c:showPercent val="0"/>
+              <c:showBubbleSize val="0"/>
+              <c:extLst>
+                <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
+                  <c15:dlblFieldTable/>
+                  <c15:xForSave val="1"/>
+                  <c15:showDataLabelsRange val="1"/>
+                </c:ext>
+                <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                  <c16:uniqueId val="{00000004-89D1-E846-B27A-3DA1AEF5883E}"/>
+                </c:ext>
+              </c:extLst>
+            </c:dLbl>
+            <c:dLbl>
+              <c:idx val="4"/>
+              <c:tx>
+                <c:rich>
+                  <a:bodyPr/>
+                  <a:lstStyle/>
+                  <a:p>
+                    <a:fld id="{98171EE7-B3A9-A146-9FC1-D39C5FFB3085}" type="CELLRANGE">
+                      <a:rPr lang="en-US"/>
+                      <a:pPr/>
+                      <a:t>[CELLRANGE]</a:t>
+                    </a:fld>
+                    <a:endParaRPr lang="en-US"/>
+                  </a:p>
+                </c:rich>
+              </c:tx>
+              <c:showLegendKey val="0"/>
+              <c:showVal val="0"/>
+              <c:showCatName val="0"/>
+              <c:showSerName val="0"/>
+              <c:showPercent val="0"/>
+              <c:showBubbleSize val="0"/>
+              <c:extLst>
+                <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
+                  <c15:dlblFieldTable/>
+                  <c15:xForSave val="1"/>
+                  <c15:showDataLabelsRange val="1"/>
+                </c:ext>
+                <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                  <c16:uniqueId val="{00000005-89D1-E846-B27A-3DA1AEF5883E}"/>
+                </c:ext>
+              </c:extLst>
+            </c:dLbl>
+            <c:dLbl>
+              <c:idx val="5"/>
+              <c:tx>
+                <c:rich>
+                  <a:bodyPr/>
+                  <a:lstStyle/>
+                  <a:p>
+                    <a:fld id="{DDA16D35-B1C2-9940-9D83-B47B2EE7E872}" type="CELLRANGE">
+                      <a:rPr lang="en-US"/>
+                      <a:pPr/>
+                      <a:t>[CELLRANGE]</a:t>
+                    </a:fld>
+                    <a:endParaRPr lang="en-US"/>
+                  </a:p>
+                </c:rich>
+              </c:tx>
+              <c:showLegendKey val="0"/>
+              <c:showVal val="0"/>
+              <c:showCatName val="0"/>
+              <c:showSerName val="0"/>
+              <c:showPercent val="0"/>
+              <c:showBubbleSize val="0"/>
+              <c:extLst>
+                <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
+                  <c15:dlblFieldTable/>
+                  <c15:xForSave val="1"/>
+                  <c15:showDataLabelsRange val="1"/>
+                </c:ext>
+                <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                  <c16:uniqueId val="{00000006-89D1-E846-B27A-3DA1AEF5883E}"/>
+                </c:ext>
+              </c:extLst>
+            </c:dLbl>
+            <c:dLbl>
+              <c:idx val="6"/>
+              <c:tx>
+                <c:rich>
+                  <a:bodyPr/>
+                  <a:lstStyle/>
+                  <a:p>
+                    <a:fld id="{298D02FB-CCD7-A345-913A-52D4BAE9AA26}" type="CELLRANGE">
+                      <a:rPr lang="en-US"/>
+                      <a:pPr/>
+                      <a:t>[CELLRANGE]</a:t>
+                    </a:fld>
+                    <a:endParaRPr lang="en-US"/>
+                  </a:p>
+                </c:rich>
+              </c:tx>
+              <c:showLegendKey val="0"/>
+              <c:showVal val="0"/>
+              <c:showCatName val="0"/>
+              <c:showSerName val="0"/>
+              <c:showPercent val="0"/>
+              <c:showBubbleSize val="0"/>
+              <c:extLst>
+                <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
+                  <c15:dlblFieldTable/>
+                  <c15:xForSave val="1"/>
+                  <c15:showDataLabelsRange val="1"/>
+                </c:ext>
+                <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                  <c16:uniqueId val="{00000007-89D1-E846-B27A-3DA1AEF5883E}"/>
+                </c:ext>
+              </c:extLst>
+            </c:dLbl>
+            <c:dLbl>
+              <c:idx val="7"/>
+              <c:tx>
+                <c:rich>
+                  <a:bodyPr/>
+                  <a:lstStyle/>
+                  <a:p>
+                    <a:fld id="{DB25DE9E-BDA5-FF4D-9D3B-00BE920C02EA}" type="CELLRANGE">
+                      <a:rPr lang="en-US"/>
+                      <a:pPr/>
+                      <a:t>[CELLRANGE]</a:t>
+                    </a:fld>
+                    <a:endParaRPr lang="en-US"/>
+                  </a:p>
+                </c:rich>
+              </c:tx>
+              <c:showLegendKey val="0"/>
+              <c:showVal val="0"/>
+              <c:showCatName val="0"/>
+              <c:showSerName val="0"/>
+              <c:showPercent val="0"/>
+              <c:showBubbleSize val="0"/>
+              <c:extLst>
+                <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
+                  <c15:dlblFieldTable/>
+                  <c15:xForSave val="1"/>
+                  <c15:showDataLabelsRange val="1"/>
+                </c:ext>
+                <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                  <c16:uniqueId val="{00000008-89D1-E846-B27A-3DA1AEF5883E}"/>
+                </c:ext>
+              </c:extLst>
+            </c:dLbl>
+            <c:spPr>
+              <a:noFill/>
+              <a:ln>
+                <a:noFill/>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:txPr>
+              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
+                <a:spAutoFit/>
+              </a:bodyPr>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="tx1">
+                        <a:lumMod val="75000"/>
+                        <a:lumOff val="25000"/>
+                      </a:schemeClr>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="+mn-cs"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:endParaRPr lang="en-TR"/>
+              </a:p>
+            </c:txPr>
+            <c:showLegendKey val="0"/>
+            <c:showVal val="0"/>
+            <c:showCatName val="0"/>
+            <c:showSerName val="0"/>
+            <c:showPercent val="0"/>
+            <c:showBubbleSize val="0"/>
+            <c:showLeaderLines val="0"/>
+            <c:extLst>
+              <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
+                <c15:showDataLabelsRange val="1"/>
+                <c15:showLeaderLines val="1"/>
+                <c15:leaderLines>
+                  <c:spPr>
+                    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+                      <a:solidFill>
+                        <a:schemeClr val="tx1">
+                          <a:lumMod val="35000"/>
+                          <a:lumOff val="65000"/>
+                        </a:schemeClr>
+                      </a:solidFill>
+                      <a:round/>
+                    </a:ln>
+                    <a:effectLst/>
+                  </c:spPr>
+                </c15:leaderLines>
+              </c:ext>
+            </c:extLst>
+          </c:dLbls>
+          <c:xVal>
+            <c:numRef>
+              <c:f>Matrix!$B$2:$B$9</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="8"/>
+                <c:pt idx="0">
+                  <c:v>3</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>2</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>2</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>1</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>5</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>1</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>3</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>5</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:xVal>
+          <c:yVal>
+            <c:numRef>
+              <c:f>Matrix!$C$2:$C$9</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="8"/>
+                <c:pt idx="0">
+                  <c:v>4</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>5</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>4</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>5</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>5</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>5</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>5</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>2</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:yVal>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
+              <c15:datalabelsRange>
+                <c15:f>Matrix!$A$2:$A$9</c15:f>
+                <c15:dlblRangeCache>
+                  <c:ptCount val="8"/>
+                  <c:pt idx="0">
+                    <c:v>UC1</c:v>
+                  </c:pt>
+                  <c:pt idx="1">
+                    <c:v>UC2</c:v>
+                  </c:pt>
+                  <c:pt idx="2">
+                    <c:v>UC3</c:v>
+                  </c:pt>
+                  <c:pt idx="3">
+                    <c:v>UC4</c:v>
+                  </c:pt>
+                  <c:pt idx="4">
+                    <c:v>UC5</c:v>
+                  </c:pt>
+                  <c:pt idx="5">
+                    <c:v>UC6</c:v>
+                  </c:pt>
+                  <c:pt idx="6">
+                    <c:v>UC7</c:v>
+                  </c:pt>
+                  <c:pt idx="7">
+                    <c:v>UC8</c:v>
+                  </c:pt>
+                </c15:dlblRangeCache>
+              </c15:datalabelsRange>
+            </c:ext>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-89D1-E846-B27A-3DA1AEF5883E}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
+        <c:axId val="532152496"/>
+        <c:axId val="566513936"/>
+      </c:scatterChart>
+      <c:valAx>
+        <c:axId val="532152496"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="25000"/>
+                <a:lumOff val="75000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-TR"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="566513936"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="midCat"/>
+      </c:valAx>
+      <c:valAx>
+        <c:axId val="566513936"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="25000"/>
+                <a:lumOff val="75000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-TR"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="532152496"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="midCat"/>
+      </c:valAx>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+    </c:plotArea>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
+    <c:extLst>
+      <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
+        <c16r3:dataDisplayOptions16>
+          <c16r3:dispNaAsBlank val="1"/>
+        </c16r3:dataDisplayOptions16>
+      </c:ext>
+    </c:extLst>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:schemeClr val="bg1"/>
+    </a:solidFill>
+    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:solidFill>
+        <a:schemeClr val="tx1">
+          <a:lumMod val="15000"/>
+          <a:lumOff val="85000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:round/>
+    </a:ln>
+    <a:effectLst/>
+  </c:spPr>
+  <c:txPr>
+    <a:bodyPr/>
+    <a:lstStyle/>
+    <a:p>
+      <a:pPr>
+        <a:defRPr/>
+      </a:pPr>
+      <a:endParaRPr lang="en-TR"/>
+    </a:p>
+  </c:txPr>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
+<file path=xl/charts/colors1.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
+  <a:schemeClr val="accent1"/>
+  <a:schemeClr val="accent2"/>
+  <a:schemeClr val="accent3"/>
+  <a:schemeClr val="accent4"/>
+  <a:schemeClr val="accent5"/>
+  <a:schemeClr val="accent6"/>
+  <cs:variation/>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+    <a:lumOff val="20000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+    <a:lumOff val="40000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+    <a:lumOff val="30000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+    <a:lumOff val="50000"/>
+  </cs:variation>
+</cs:colorStyle>
+</file>
+
+<file path=xl/charts/style1.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="240">
+  <cs:axisTitle>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:axisTitle>
+  <cs:categoryAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:categoryAxis>
+  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="bg1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:chartArea>
+  <cs:dataLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="75000"/>
+        <a:lumOff val="25000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataLabel>
+  <cs:dataLabelCallout>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
+      <a:spAutoFit/>
+    </cs:bodyPr>
+  </cs:dataLabelCallout>
+  <cs:dataPoint>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint>
+  <cs:dataPoint3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint3D>
+  <cs:dataPointLine>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointLine>
+  <cs:dataPointMarker>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointMarker>
+  <cs:dataPointMarkerLayout symbol="circle" size="5"/>
+  <cs:dataPointWireframe>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointWireframe>
+  <cs:dataTable>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataTable>
+  <cs:downBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="75000"/>
+          <a:lumOff val="25000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:downBar>
+  <cs:dropLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dropLine>
+  <cs:errorBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:errorBar>
+  <cs:floor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:floor>
+  <cs:gridlineMajor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMajor>
+  <cs:gridlineMinor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="5000"/>
+            <a:lumOff val="95000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMinor>
+  <cs:hiLoLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="50000"/>
+            <a:lumOff val="50000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:hiLoLine>
+  <cs:leaderLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:leaderLine>
+  <cs:legend>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:legend>
+  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea>
+  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea3D>
+  <cs:seriesAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:seriesAxis>
+  <cs:seriesLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:seriesLine>
+  <cs:title>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1400" b="0" kern="1200" spc="0" baseline="0"/>
+  </cs:title>
+  <cs:trendline>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:prstDash val="sysDot"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:trendline>
+  <cs:trendlineLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:trendlineLabel>
+  <cs:upBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:upBar>
+  <cs:valueAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:valueAxis>
+  <cs:wall>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:wall>
+</cs:chartStyle>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>793750</xdr:colOff>
+      <xdr:row>11</xdr:row>
+      <xdr:rowOff>158750</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>13</xdr:col>
+      <xdr:colOff>412750</xdr:colOff>
+      <xdr:row>26</xdr:row>
+      <xdr:rowOff>44450</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="2" name="Chart 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{B735633B-FF53-21BD-0711-C7082573CFC3}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1132,7 +2433,7 @@
       </c>
     </row>
   </sheetData>
-  <dataValidations count="2">
+  <dataValidations disablePrompts="1" count="2">
     <dataValidation type="whole" showErrorMessage="1" errorTitle="Score 1-5" error="Please enter a whole number from 1 to 5." sqref="H2:K9" xr:uid="{00000000-0002-0000-0000-000000000000}">
       <formula1>1</formula1>
       <formula2>5</formula2>
@@ -1149,6 +2450,143 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{70269925-E3F4-B049-BA03-E1767B4A947B}">
+  <dimension ref="A1:C9"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="3" max="3" width="12.6640625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>74</v>
+      </c>
+      <c r="C1" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A2" t="str">
+        <f>'Use Cases'!A2</f>
+        <v>UC1</v>
+      </c>
+      <c r="B2">
+        <f>'Use Cases'!J2</f>
+        <v>3</v>
+      </c>
+      <c r="C2">
+        <f>'Use Cases'!H2</f>
+        <v>4</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A3" t="str">
+        <f>'Use Cases'!A3</f>
+        <v>UC2</v>
+      </c>
+      <c r="B3">
+        <f>'Use Cases'!J3</f>
+        <v>2</v>
+      </c>
+      <c r="C3">
+        <f>'Use Cases'!H3</f>
+        <v>5</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A4" t="str">
+        <f>'Use Cases'!A4</f>
+        <v>UC3</v>
+      </c>
+      <c r="B4">
+        <f>'Use Cases'!J4</f>
+        <v>2</v>
+      </c>
+      <c r="C4">
+        <f>'Use Cases'!H4</f>
+        <v>4</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A5" t="str">
+        <f>'Use Cases'!A5</f>
+        <v>UC4</v>
+      </c>
+      <c r="B5">
+        <f>'Use Cases'!J5</f>
+        <v>1</v>
+      </c>
+      <c r="C5">
+        <f>'Use Cases'!H5</f>
+        <v>5</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A6" t="str">
+        <f>'Use Cases'!A6</f>
+        <v>UC5</v>
+      </c>
+      <c r="B6">
+        <f>'Use Cases'!J6</f>
+        <v>5</v>
+      </c>
+      <c r="C6">
+        <f>'Use Cases'!H6</f>
+        <v>5</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A7" t="str">
+        <f>'Use Cases'!A7</f>
+        <v>UC6</v>
+      </c>
+      <c r="B7">
+        <f>'Use Cases'!J7</f>
+        <v>1</v>
+      </c>
+      <c r="C7">
+        <f>'Use Cases'!H7</f>
+        <v>5</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A8" t="str">
+        <f>'Use Cases'!A8</f>
+        <v>UC7</v>
+      </c>
+      <c r="B8">
+        <f>'Use Cases'!J8</f>
+        <v>3</v>
+      </c>
+      <c r="C8">
+        <f>'Use Cases'!H8</f>
+        <v>5</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A9" t="str">
+        <f>'Use Cases'!A9</f>
+        <v>UC8</v>
+      </c>
+      <c r="B9">
+        <f>'Use Cases'!J9</f>
+        <v>5</v>
+      </c>
+      <c r="C9">
+        <f>'Use Cases'!H9</f>
+        <v>2</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:F9"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>

</xml_diff>

<commit_message>
M5 step 7: 2x2 matrix - axes cross at 3, labels low, chart and axis titles
</commit_message>
<xml_diff>
--- a/excel/AI_Use_Case_Prioritization.xlsx
+++ b/excel/AI_Use_Case_Prioritization.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/mac1/Desktop/app_projects/supplier-data-health-check/excel/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D76D9421-045E-6444-8C06-913A80401EDB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AA3365F8-7757-EA43-A761-E61A947C02BE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="16260" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -412,6 +412,32 @@
   </mc:AlternateContent>
   <c:chart>
     <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="en-US" sz="1400" b="0" i="0" u="none" strike="noStrike" baseline="0"/>
+              <a:t>AI use cases: value vs. effort</a:t>
+            </a:r>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:rich>
+      </c:tx>
       <c:overlay val="0"/>
       <c:spPr>
         <a:noFill/>
@@ -491,7 +517,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{AE28D843-2E10-8D4B-B511-6E5BD9871D2E}" type="CELLRANGE">
+                    <a:fld id="{FAC1187A-EC9F-524F-9A21-081F3A46B2FC}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -524,7 +550,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{C5B6A356-D241-8F4B-896C-8B0132F7D7E1}" type="CELLRANGE">
+                    <a:fld id="{356779A8-3FCB-4948-9C59-7762F0BEF91E}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -557,7 +583,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{A192A440-33E3-4848-B253-46A9D2677265}" type="CELLRANGE">
+                    <a:fld id="{F71318F1-79FD-5945-8884-A77004D0391C}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -590,7 +616,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{E2707DB1-2CC9-5046-B13E-9112D8CBEA8A}" type="CELLRANGE">
+                    <a:fld id="{C42EE15F-B05E-8F42-B72D-9847C443E95D}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -623,7 +649,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{98171EE7-B3A9-A146-9FC1-D39C5FFB3085}" type="CELLRANGE">
+                    <a:fld id="{9762BC34-AC3C-E54C-9DFD-2E6C85D029F3}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -656,7 +682,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{DDA16D35-B1C2-9940-9D83-B47B2EE7E872}" type="CELLRANGE">
+                    <a:fld id="{FFD9B6C6-E556-B444-B696-6C3916F19971}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -689,7 +715,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{298D02FB-CCD7-A345-913A-52D4BAE9AA26}" type="CELLRANGE">
+                    <a:fld id="{A14A02CC-240D-4B42-BA40-8B43A1CFDE88}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -722,7 +748,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{DB25DE9E-BDA5-FF4D-9D3B-00BE920C02EA}" type="CELLRANGE">
+                    <a:fld id="{EA1310D9-0ECD-9240-8372-AE0DC881AB34}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -942,10 +968,74 @@
             <a:effectLst/>
           </c:spPr>
         </c:majorGridlines>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="tx1">
+                        <a:lumMod val="65000"/>
+                        <a:lumOff val="35000"/>
+                      </a:schemeClr>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="+mn-cs"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:r>
+                  <a:rPr lang="en-US" sz="1000" b="0" i="0" u="none" strike="noStrike" baseline="0"/>
+                  <a:t>Effort (1 = days, 5 = months)</a:t>
+                </a:r>
+                <a:endParaRPr lang="en-US"/>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:layout>
+            <c:manualLayout>
+              <c:xMode val="edge"/>
+              <c:yMode val="edge"/>
+              <c:x val="0.37015157480314959"/>
+              <c:y val="0.90645815106445027"/>
+            </c:manualLayout>
+          </c:layout>
+          <c:overlay val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:txPr>
+            <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr>
+                <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1">
+                      <a:lumMod val="65000"/>
+                      <a:lumOff val="35000"/>
+                    </a:schemeClr>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:endParaRPr lang="en-TR"/>
+            </a:p>
+          </c:txPr>
+        </c:title>
         <c:numFmt formatCode="General" sourceLinked="1"/>
         <c:majorTickMark val="none"/>
         <c:minorTickMark val="none"/>
-        <c:tickLblPos val="nextTo"/>
+        <c:tickLblPos val="low"/>
         <c:spPr>
           <a:noFill/>
           <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
@@ -980,7 +1070,7 @@
           </a:p>
         </c:txPr>
         <c:crossAx val="566513936"/>
-        <c:crosses val="autoZero"/>
+        <c:crossesAt val="3"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
       <c:valAx>
@@ -1004,10 +1094,77 @@
             <a:effectLst/>
           </c:spPr>
         </c:majorGridlines>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr rot="-5400000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="tx1">
+                        <a:lumMod val="65000"/>
+                        <a:lumOff val="35000"/>
+                      </a:schemeClr>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="+mn-cs"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:r>
+                  <a:rPr lang="en-US" sz="1000" b="0" i="0" u="none" strike="noStrike" baseline="0"/>
+                  <a:t>Business value (1-5)</a:t>
+                </a:r>
+                <a:r>
+                  <a:rPr lang="en-US"/>
+                  <a:t> </a:t>
+                </a:r>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:layout>
+            <c:manualLayout>
+              <c:xMode val="edge"/>
+              <c:yMode val="edge"/>
+              <c:x val="1.6666666666666666E-2"/>
+              <c:y val="0.28733012540099157"/>
+            </c:manualLayout>
+          </c:layout>
+          <c:overlay val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:txPr>
+            <a:bodyPr rot="-5400000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr>
+                <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1">
+                      <a:lumMod val="65000"/>
+                      <a:lumOff val="35000"/>
+                    </a:schemeClr>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:endParaRPr lang="en-TR"/>
+            </a:p>
+          </c:txPr>
+        </c:title>
         <c:numFmt formatCode="General" sourceLinked="1"/>
         <c:majorTickMark val="none"/>
         <c:minorTickMark val="none"/>
-        <c:tickLblPos val="nextTo"/>
+        <c:tickLblPos val="low"/>
         <c:spPr>
           <a:noFill/>
           <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
@@ -1042,7 +1199,7 @@
           </a:p>
         </c:txPr>
         <c:crossAx val="532152496"/>
-        <c:crosses val="autoZero"/>
+        <c:crossesAt val="3"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
       <c:spPr>

</xml_diff>

<commit_message>
M5 step 8: quadrant names (Quick wins, Big projects, Fill-ins, Avoid) and chart exported as PNG
</commit_message>
<xml_diff>
--- a/excel/AI_Use_Case_Prioritization.xlsx
+++ b/excel/AI_Use_Case_Prioritization.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/mac1/Desktop/app_projects/supplier-data-health-check/excel/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AA3365F8-7757-EA43-A761-E61A947C02BE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6F2E09DF-BF79-0243-BA99-2AFCC7D933D6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="16260" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -517,7 +517,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{FAC1187A-EC9F-524F-9A21-081F3A46B2FC}" type="CELLRANGE">
+                    <a:fld id="{C04D5A38-9083-4D49-A8D5-34A28AA73A12}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -550,7 +550,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{356779A8-3FCB-4948-9C59-7762F0BEF91E}" type="CELLRANGE">
+                    <a:fld id="{E5AB3BBC-B41A-A646-96D3-CE17761A0BFA}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -583,7 +583,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{F71318F1-79FD-5945-8884-A77004D0391C}" type="CELLRANGE">
+                    <a:fld id="{D4D2D53E-DED1-4740-8352-2A199C24A486}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -616,7 +616,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{C42EE15F-B05E-8F42-B72D-9847C443E95D}" type="CELLRANGE">
+                    <a:fld id="{DE754A7E-2E34-F341-B510-C488EFA26B80}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -649,7 +649,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{9762BC34-AC3C-E54C-9DFD-2E6C85D029F3}" type="CELLRANGE">
+                    <a:fld id="{BF18A3B6-5D05-B74B-9EFA-C75F7B4A30BB}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -682,7 +682,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{FFD9B6C6-E556-B444-B696-6C3916F19971}" type="CELLRANGE">
+                    <a:fld id="{5D458BF3-1E99-E745-885C-D29C54BE86E6}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -715,7 +715,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{A14A02CC-240D-4B42-BA40-8B43A1CFDE88}" type="CELLRANGE">
+                    <a:fld id="{5C8A02EE-4415-1344-B80A-69BF2475A51D}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -748,7 +748,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{EA1310D9-0ECD-9240-8372-AE0DC881AB34}" type="CELLRANGE">
+                    <a:fld id="{9BDBCB24-BF27-8E43-A927-FBA24734301F}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -1251,6 +1251,7 @@
     <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
     <c:pageSetup/>
   </c:printSettings>
+  <c:userShapes r:id="rId3"/>
 </c:chartSpace>
 </file>
 
@@ -1814,16 +1815,16 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>7</xdr:col>
-      <xdr:colOff>793750</xdr:colOff>
-      <xdr:row>11</xdr:row>
-      <xdr:rowOff>158750</xdr:rowOff>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>800100</xdr:colOff>
+      <xdr:row>8</xdr:row>
+      <xdr:rowOff>165100</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>13</xdr:col>
-      <xdr:colOff>412750</xdr:colOff>
-      <xdr:row>26</xdr:row>
-      <xdr:rowOff>44450</xdr:rowOff>
+      <xdr:colOff>622300</xdr:colOff>
+      <xdr:row>28</xdr:row>
+      <xdr:rowOff>152400</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
@@ -1849,6 +1850,420 @@
     <xdr:clientData/>
   </xdr:twoCellAnchor>
 </xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
+<c:userShapes xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <cdr:relSizeAnchor xmlns:cdr="http://schemas.openxmlformats.org/drawingml/2006/chartDrawing">
+    <cdr:from>
+      <cdr:x>0.01528</cdr:x>
+      <cdr:y>0.05324</cdr:y>
+    </cdr:from>
+    <cdr:to>
+      <cdr:x>0.21528</cdr:x>
+      <cdr:y>0.38657</cdr:y>
+    </cdr:to>
+    <cdr:sp macro="" textlink="">
+      <cdr:nvSpPr>
+        <cdr:cNvPr id="2" name="TextBox 1">
+          <a:extLst xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{ADC94912-D5A1-8747-427F-160C6F2FDC12}"/>
+            </a:ext>
+          </a:extLst>
+        </cdr:cNvPr>
+        <cdr:cNvSpPr txBox="1"/>
+      </cdr:nvSpPr>
+      <cdr:spPr>
+        <a:xfrm xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:off x="69850" y="146050"/>
+          <a:ext cx="914400" cy="914400"/>
+        </a:xfrm>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </cdr:spPr>
+      <cdr:txBody>
+        <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" vertOverflow="clip" wrap="none" rtlCol="0"/>
+        <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:endParaRPr lang="en-US" sz="1100" kern="1200"/>
+        </a:p>
+      </cdr:txBody>
+    </cdr:sp>
+  </cdr:relSizeAnchor>
+  <cdr:relSizeAnchor xmlns:cdr="http://schemas.openxmlformats.org/drawingml/2006/chartDrawing">
+    <cdr:from>
+      <cdr:x>0.0125</cdr:x>
+      <cdr:y>0.03009</cdr:y>
+    </cdr:from>
+    <cdr:to>
+      <cdr:x>0.19861</cdr:x>
+      <cdr:y>0.11806</cdr:y>
+    </cdr:to>
+    <cdr:sp macro="" textlink="">
+      <cdr:nvSpPr>
+        <cdr:cNvPr id="3" name="TextBox 2">
+          <a:extLst xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{BF356A50-A119-4E2E-172B-6D83EB80FE12}"/>
+            </a:ext>
+          </a:extLst>
+        </cdr:cNvPr>
+        <cdr:cNvSpPr txBox="1"/>
+      </cdr:nvSpPr>
+      <cdr:spPr>
+        <a:xfrm xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:off x="57150" y="82550"/>
+          <a:ext cx="850900" cy="241300"/>
+        </a:xfrm>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </cdr:spPr>
+      <cdr:txBody>
+        <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" vertOverflow="clip" wrap="none" rtlCol="0"/>
+        <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:r>
+            <a:rPr lang="en-US" b="1"/>
+            <a:t>Quick wins</a:t>
+          </a:r>
+          <a:endParaRPr lang="en-US" sz="1100" b="1" kern="1200"/>
+        </a:p>
+      </cdr:txBody>
+    </cdr:sp>
+  </cdr:relSizeAnchor>
+  <cdr:relSizeAnchor xmlns:cdr="http://schemas.openxmlformats.org/drawingml/2006/chartDrawing">
+    <cdr:from>
+      <cdr:x>0.8</cdr:x>
+      <cdr:y>0.03472</cdr:y>
+    </cdr:from>
+    <cdr:to>
+      <cdr:x>0.97639</cdr:x>
+      <cdr:y>0.12731</cdr:y>
+    </cdr:to>
+    <cdr:sp macro="" textlink="">
+      <cdr:nvSpPr>
+        <cdr:cNvPr id="4" name="TextBox 3">
+          <a:extLst xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{5B8A6C22-6671-BE70-9635-C4322F1C7485}"/>
+            </a:ext>
+          </a:extLst>
+        </cdr:cNvPr>
+        <cdr:cNvSpPr txBox="1"/>
+      </cdr:nvSpPr>
+      <cdr:spPr>
+        <a:xfrm xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:off x="3657600" y="95250"/>
+          <a:ext cx="806450" cy="254000"/>
+        </a:xfrm>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </cdr:spPr>
+      <cdr:txBody>
+        <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" vertOverflow="clip" wrap="none" rtlCol="0"/>
+        <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:r>
+            <a:rPr lang="en-US" b="1"/>
+            <a:t>Big projects</a:t>
+          </a:r>
+          <a:endParaRPr lang="en-US" sz="1100" b="1" kern="1200"/>
+        </a:p>
+      </cdr:txBody>
+    </cdr:sp>
+  </cdr:relSizeAnchor>
+  <cdr:relSizeAnchor xmlns:cdr="http://schemas.openxmlformats.org/drawingml/2006/chartDrawing">
+    <cdr:from>
+      <cdr:x>0.0125</cdr:x>
+      <cdr:y>0.90509</cdr:y>
+    </cdr:from>
+    <cdr:to>
+      <cdr:x>0.2125</cdr:x>
+      <cdr:y>1</cdr:y>
+    </cdr:to>
+    <cdr:sp macro="" textlink="">
+      <cdr:nvSpPr>
+        <cdr:cNvPr id="5" name="TextBox 4">
+          <a:extLst xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{F9FFE39B-7D76-E6DE-6214-728F2F767CD7}"/>
+            </a:ext>
+          </a:extLst>
+        </cdr:cNvPr>
+        <cdr:cNvSpPr txBox="1"/>
+      </cdr:nvSpPr>
+      <cdr:spPr>
+        <a:xfrm xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:off x="57150" y="2482850"/>
+          <a:ext cx="914400" cy="260350"/>
+        </a:xfrm>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </cdr:spPr>
+      <cdr:txBody>
+        <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" vertOverflow="clip" wrap="none" rtlCol="0"/>
+        <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:endParaRPr lang="en-US" sz="1100" kern="1200"/>
+        </a:p>
+      </cdr:txBody>
+    </cdr:sp>
+  </cdr:relSizeAnchor>
+  <cdr:relSizeAnchor xmlns:cdr="http://schemas.openxmlformats.org/drawingml/2006/chartDrawing">
+    <cdr:from>
+      <cdr:x>0.00972</cdr:x>
+      <cdr:y>0.87269</cdr:y>
+    </cdr:from>
+    <cdr:to>
+      <cdr:x>0.21806</cdr:x>
+      <cdr:y>1</cdr:y>
+    </cdr:to>
+    <cdr:sp macro="" textlink="">
+      <cdr:nvSpPr>
+        <cdr:cNvPr id="6" name="TextBox 5">
+          <a:extLst xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{FA5C7D2A-35A5-114A-5471-6E2D5567E8D1}"/>
+            </a:ext>
+          </a:extLst>
+        </cdr:cNvPr>
+        <cdr:cNvSpPr txBox="1"/>
+      </cdr:nvSpPr>
+      <cdr:spPr>
+        <a:xfrm xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:off x="44450" y="2393950"/>
+          <a:ext cx="952500" cy="349250"/>
+        </a:xfrm>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </cdr:spPr>
+      <cdr:txBody>
+        <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" vertOverflow="clip" wrap="none" rtlCol="0"/>
+        <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:endParaRPr lang="en-US" sz="1100" kern="1200"/>
+        </a:p>
+      </cdr:txBody>
+    </cdr:sp>
+  </cdr:relSizeAnchor>
+  <cdr:relSizeAnchor xmlns:cdr="http://schemas.openxmlformats.org/drawingml/2006/chartDrawing">
+    <cdr:from>
+      <cdr:x>0.01111</cdr:x>
+      <cdr:y>0.88889</cdr:y>
+    </cdr:from>
+    <cdr:to>
+      <cdr:x>0.19722</cdr:x>
+      <cdr:y>0.97685</cdr:y>
+    </cdr:to>
+    <cdr:sp macro="" textlink="">
+      <cdr:nvSpPr>
+        <cdr:cNvPr id="7" name="TextBox 1">
+          <a:extLst xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{65A3D45E-CF07-A999-FE46-6DABEC2BC8BD}"/>
+            </a:ext>
+          </a:extLst>
+        </cdr:cNvPr>
+        <cdr:cNvSpPr txBox="1"/>
+      </cdr:nvSpPr>
+      <cdr:spPr>
+        <a:xfrm xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:off x="50800" y="2438400"/>
+          <a:ext cx="850900" cy="241300"/>
+        </a:xfrm>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </cdr:spPr>
+      <cdr:txBody>
+        <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="none" rtlCol="0"/>
+        <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:lvl1pPr marL="0" indent="0">
+            <a:defRPr sz="1100">
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:lvl1pPr>
+          <a:lvl2pPr marL="457200" indent="0">
+            <a:defRPr sz="1100">
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:lvl2pPr>
+          <a:lvl3pPr marL="914400" indent="0">
+            <a:defRPr sz="1100">
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:lvl3pPr>
+          <a:lvl4pPr marL="1371600" indent="0">
+            <a:defRPr sz="1100">
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:lvl4pPr>
+          <a:lvl5pPr marL="1828800" indent="0">
+            <a:defRPr sz="1100">
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:lvl5pPr>
+          <a:lvl6pPr marL="2286000" indent="0">
+            <a:defRPr sz="1100">
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:lvl6pPr>
+          <a:lvl7pPr marL="2743200" indent="0">
+            <a:defRPr sz="1100">
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:lvl7pPr>
+          <a:lvl8pPr marL="3200400" indent="0">
+            <a:defRPr sz="1100">
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:lvl8pPr>
+          <a:lvl9pPr marL="3657600" indent="0">
+            <a:defRPr sz="1100">
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:lvl9pPr>
+        </a:lstStyle>
+        <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:r>
+            <a:rPr lang="en-US" sz="1100" b="1" kern="1200"/>
+            <a:t>Fill-ins</a:t>
+          </a:r>
+        </a:p>
+      </cdr:txBody>
+    </cdr:sp>
+  </cdr:relSizeAnchor>
+  <cdr:relSizeAnchor xmlns:cdr="http://schemas.openxmlformats.org/drawingml/2006/chartDrawing">
+    <cdr:from>
+      <cdr:x>0.81389</cdr:x>
+      <cdr:y>0.89815</cdr:y>
+    </cdr:from>
+    <cdr:to>
+      <cdr:x>1</cdr:x>
+      <cdr:y>0.98611</cdr:y>
+    </cdr:to>
+    <cdr:sp macro="" textlink="">
+      <cdr:nvSpPr>
+        <cdr:cNvPr id="8" name="TextBox 1">
+          <a:extLst xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{B89690C8-93CF-22A0-ED20-F68252A01C8A}"/>
+            </a:ext>
+          </a:extLst>
+        </cdr:cNvPr>
+        <cdr:cNvSpPr txBox="1"/>
+      </cdr:nvSpPr>
+      <cdr:spPr>
+        <a:xfrm xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:off x="3721100" y="2463800"/>
+          <a:ext cx="850900" cy="241300"/>
+        </a:xfrm>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </cdr:spPr>
+      <cdr:txBody>
+        <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="none" rtlCol="0"/>
+        <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:lvl1pPr marL="0" indent="0">
+            <a:defRPr sz="1100">
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:lvl1pPr>
+          <a:lvl2pPr marL="457200" indent="0">
+            <a:defRPr sz="1100">
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:lvl2pPr>
+          <a:lvl3pPr marL="914400" indent="0">
+            <a:defRPr sz="1100">
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:lvl3pPr>
+          <a:lvl4pPr marL="1371600" indent="0">
+            <a:defRPr sz="1100">
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:lvl4pPr>
+          <a:lvl5pPr marL="1828800" indent="0">
+            <a:defRPr sz="1100">
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:lvl5pPr>
+          <a:lvl6pPr marL="2286000" indent="0">
+            <a:defRPr sz="1100">
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:lvl6pPr>
+          <a:lvl7pPr marL="2743200" indent="0">
+            <a:defRPr sz="1100">
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:lvl7pPr>
+          <a:lvl8pPr marL="3200400" indent="0">
+            <a:defRPr sz="1100">
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:lvl8pPr>
+          <a:lvl9pPr marL="3657600" indent="0">
+            <a:defRPr sz="1100">
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:lvl9pPr>
+        </a:lstStyle>
+        <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:r>
+            <a:rPr lang="en-US" b="1"/>
+            <a:t>Avoid</a:t>
+          </a:r>
+          <a:endParaRPr lang="en-US" sz="1100" b="1" kern="1200"/>
+        </a:p>
+      </cdr:txBody>
+    </cdr:sp>
+  </cdr:relSizeAnchor>
+</c:userShapes>
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>

</xml_diff>

<commit_message>
M5 step 9: clearer quadrant lines and combined UC4/UC6 label
</commit_message>
<xml_diff>
--- a/excel/AI_Use_Case_Prioritization.xlsx
+++ b/excel/AI_Use_Case_Prioritization.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/mac1/Desktop/app_projects/supplier-data-health-check/excel/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6F2E09DF-BF79-0243-BA99-2AFCC7D933D6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FA3850EC-81E1-0E41-91E7-D89BFA844DF8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="16260" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -517,7 +517,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{C04D5A38-9083-4D49-A8D5-34A28AA73A12}" type="CELLRANGE">
+                    <a:fld id="{619AA6B9-46B6-8644-811D-4D288DAA9BE2}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -550,7 +550,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{E5AB3BBC-B41A-A646-96D3-CE17761A0BFA}" type="CELLRANGE">
+                    <a:fld id="{FD5AEAC8-5802-FF49-986A-FD128111043C}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -583,7 +583,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{D4D2D53E-DED1-4740-8352-2A199C24A486}" type="CELLRANGE">
+                    <a:fld id="{0BC4671C-F9C5-D845-B71D-60B5D59E72C6}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -616,11 +616,10 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{DE754A7E-2E34-F341-B510-C488EFA26B80}" type="CELLRANGE">
-                      <a:rPr lang="en-US"/>
-                      <a:pPr/>
-                      <a:t>[CELLRANGE]</a:t>
-                    </a:fld>
+                    <a:r>
+                      <a:rPr lang="en-US" sz="900" b="0" i="0" u="none" strike="noStrike" baseline="0"/>
+                      <a:t>UC4 / UC6</a:t>
+                    </a:r>
                     <a:endParaRPr lang="en-US"/>
                   </a:p>
                 </c:rich>
@@ -633,8 +632,6 @@
               <c:showBubbleSize val="0"/>
               <c:extLst>
                 <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
-                  <c15:dlblFieldTable/>
-                  <c15:xForSave val="1"/>
                   <c15:showDataLabelsRange val="1"/>
                 </c:ext>
                 <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
@@ -649,7 +646,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{BF18A3B6-5D05-B74B-9EFA-C75F7B4A30BB}" type="CELLRANGE">
+                    <a:fld id="{6A8B9939-9C10-1F42-B5FF-517D71525143}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -677,32 +674,9 @@
             </c:dLbl>
             <c:dLbl>
               <c:idx val="5"/>
-              <c:tx>
-                <c:rich>
-                  <a:bodyPr/>
-                  <a:lstStyle/>
-                  <a:p>
-                    <a:fld id="{5D458BF3-1E99-E745-885C-D29C54BE86E6}" type="CELLRANGE">
-                      <a:rPr lang="en-US"/>
-                      <a:pPr/>
-                      <a:t>[CELLRANGE]</a:t>
-                    </a:fld>
-                    <a:endParaRPr lang="en-US"/>
-                  </a:p>
-                </c:rich>
-              </c:tx>
-              <c:showLegendKey val="0"/>
-              <c:showVal val="0"/>
-              <c:showCatName val="0"/>
-              <c:showSerName val="0"/>
-              <c:showPercent val="0"/>
-              <c:showBubbleSize val="0"/>
+              <c:delete val="1"/>
               <c:extLst>
-                <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
-                  <c15:dlblFieldTable/>
-                  <c15:xForSave val="1"/>
-                  <c15:showDataLabelsRange val="1"/>
-                </c:ext>
+                <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
                 <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
                   <c16:uniqueId val="{00000006-89D1-E846-B27A-3DA1AEF5883E}"/>
                 </c:ext>
@@ -715,7 +689,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{5C8A02EE-4415-1344-B80A-69BF2475A51D}" type="CELLRANGE">
+                    <a:fld id="{23243D77-6161-5048-BB46-8F0C57771F12}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -748,7 +722,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{9BDBCB24-BF27-8E43-A927-FBA24734301F}" type="CELLRANGE">
+                    <a:fld id="{92E6F524-DD09-DC45-A190-591E43388C98}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -1038,12 +1012,9 @@
         <c:tickLblPos val="low"/>
         <c:spPr>
           <a:noFill/>
-          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+          <a:ln w="19050" cap="flat" cmpd="sng" algn="ctr">
             <a:solidFill>
-              <a:schemeClr val="tx1">
-                <a:lumMod val="25000"/>
-                <a:lumOff val="75000"/>
-              </a:schemeClr>
+              <a:schemeClr val="tx1"/>
             </a:solidFill>
             <a:round/>
           </a:ln>
@@ -1167,12 +1138,9 @@
         <c:tickLblPos val="low"/>
         <c:spPr>
           <a:noFill/>
-          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+          <a:ln w="19050" cap="flat" cmpd="sng" algn="ctr">
             <a:solidFill>
-              <a:schemeClr val="tx1">
-                <a:lumMod val="25000"/>
-                <a:lumOff val="75000"/>
-              </a:schemeClr>
+              <a:schemeClr val="tx1"/>
             </a:solidFill>
             <a:round/>
           </a:ln>

</xml_diff>